<commit_message>
updated config and umm, dataset results, and triage module
</commit_message>
<xml_diff>
--- a/notebook/dataset/Triage-Module-Evaluation-Dataset.xlsx
+++ b/notebook/dataset/Triage-Module-Evaluation-Dataset.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9000"/>
+    <workbookView windowWidth="28800" windowHeight="11580"/>
   </bookViews>
   <sheets>
     <sheet name="eval" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="589" uniqueCount="290">
   <si>
     <t>prompts</t>
   </si>
@@ -48,7 +48,7 @@
     <t>Tagalog</t>
   </si>
   <si>
-    <t>Hindi ako pinayagan mag-day off ng amo ko for 3 months na.</t>
+    <t>Hindi ako pinayagan mag-day off ng amo ko for 3 buwan na.</t>
   </si>
   <si>
     <t>May karapatan ba akong magreklamo kapag sinasaktan ako ng alaga ko?</t>
@@ -102,7 +102,7 @@
     <t>Pinatutulog ako sa kitchen floor, pwede ba ireklamo yun?</t>
   </si>
   <si>
-    <t>Delayed ng 2 buwan ang sahod ko, ano po ang rights ko?</t>
+    <t>Delayed ng 2 buwan ang sahod ko, ano po kaya ang rights ko?</t>
   </si>
   <si>
     <t>Ayaw pirmahan ng amo ko ang release paper ko.</t>
@@ -129,7 +129,7 @@
     <t>Ano ang parusa sa illegal recruitment?</t>
   </si>
   <si>
-    <t>Kasama ba sa kontrata ang free food at accommodation?</t>
+    <t>Kasama ba sa kontrata ang libreng pakain at accommodation?</t>
   </si>
   <si>
     <t>Pwede bang mag-demand ng overtime pay ang domestic helper?</t>
@@ -195,49 +195,49 @@
     <t>Gusto kong malaman ang status ng kaso ko sa NLRC.</t>
   </si>
   <si>
-    <t>Attorney, valid ba ang termination if through text lang sinabi?</t>
+    <t>Attorney, is it valid ang termination if through text lang sinabi?</t>
   </si>
   <si>
     <t>Taglish</t>
   </si>
   <si>
-    <t>Nag-overstay ako ng 2 days, magkakaproblema ba ako sa Immigration?</t>
-  </si>
-  <si>
-    <t>Yung employer ko, ayaw ibigay yung separation pay ko, what to do?</t>
-  </si>
-  <si>
-    <t>Paki-check naman po kung legit itong agency na kausap ko.</t>
-  </si>
-  <si>
-    <t>Required ba magbayad ng tax sa Pinas if OFW ako?</t>
-  </si>
-  <si>
-    <t>Help po, na-harass ako ng employer ko verbally, pwede ba mag-reklamo?</t>
-  </si>
-  <si>
-    <t>Please advise, gusto ko na mag-break ng contract kasi toxic na.</t>
-  </si>
-  <si>
-    <t>Wala silang binibigay na food allowance, is that legal?</t>
+    <t>nag-overstayed me ng dalawang araw, is it a big deal ba sa Immigration?</t>
+  </si>
+  <si>
+    <t>Yung employer ko, does not wanna give yung separation pay ko, what to do?</t>
+  </si>
+  <si>
+    <t>please-check naman po kung legit itong agency na kausap ko.</t>
+  </si>
+  <si>
+    <t>is it Required ba magbayad ng tax sa Pinas if OFW ako?</t>
+  </si>
+  <si>
+    <t>Help po, na-harass ako ng employer ko verbally, pwede ba mag-reklamoto any authorities?</t>
+  </si>
+  <si>
+    <t>Please advise, gusto ko na mag-break ng contract kasi toxic na po here sa work environment.</t>
+  </si>
+  <si>
+    <t>Wala silang binibigay na food allowance im concerned, is that legal?</t>
   </si>
   <si>
     <t>My employer confiscated my phone, bawal po ba yun?</t>
   </si>
   <si>
-    <t>Pwede ba mag-file ng case sa Hong Kong Labour Department directly?</t>
-  </si>
-  <si>
-    <t>Paano i-claim ang Long Service Payment if 5 years na ako?</t>
-  </si>
-  <si>
-    <t>Nawala ko yung passport ko, paano ako makakauwi?</t>
-  </si>
-  <si>
-    <t>Need ba ng medical certificate kapag magrerenew ng contract?</t>
-  </si>
-  <si>
-    <t>Yung agency ko nanghihingi ng extra fee, scam ba 'to?</t>
+    <t>Pwede po ba mag-file ng case in Hong Kong Labour Department directly and how po?</t>
+  </si>
+  <si>
+    <t>how can i claim the Long Service Payment if 5 years na ako working in my job?</t>
+  </si>
+  <si>
+    <t>I lost my passport last night, paano ako makakauwi?</t>
+  </si>
+  <si>
+    <t>Need ba ng medical certificate for renewing my contract of employment?</t>
+  </si>
+  <si>
+    <t>Yung agency ko is asking an extra fee, scam ba 'to?</t>
   </si>
   <si>
     <t>Legal ba if bawasan yung sweldo ko due to pandemic?</t>
@@ -246,13 +246,13 @@
     <t>Can I transfer to another employer kapag na-terminate ako?</t>
   </si>
   <si>
-    <t>Ayaw nila ibigay yung plane ticket ko pauwi, what are my rights?</t>
-  </si>
-  <si>
-    <t>May pending case ako sa Pinas, makakaalis ba ako?</t>
-  </si>
-  <si>
-    <t>Sabi ng amo ko, I have to work on Sundays, bawal di ba?</t>
+    <t>the refuse to give yung plane ticket ko pauwi, what are my rights?</t>
+  </si>
+  <si>
+    <t>May pending case ako sa Pinas, will the bureau allow me to leave?</t>
+  </si>
+  <si>
+    <t>Sabi ng amo ko, I have to work on Sundays , bawal po ata yun atty what should i do po?</t>
   </si>
   <si>
     <t>Paano mag-apply ng OEC online, down kasi yung website.</t>
@@ -261,46 +261,46 @@
     <t>If ma-deport ako, can I still work in other countries?</t>
   </si>
   <si>
-    <t>Binawasan nila salary ko for electricity, tama ba yun?</t>
-  </si>
-  <si>
-    <t>Pwede ba humingi ng assistance sa OWWA for legal battle?</t>
+    <t>they reduced my salary ko for the electricity na ginamit ko, tama ba yun?</t>
+  </si>
+  <si>
+    <t>is it allowed po ba humingi ng assistance sa OWWA for legal dispute-resolution?</t>
   </si>
   <si>
     <t>Pinagbintangan ako na magnanakaw without proof, pwede ba mag-sue?</t>
   </si>
   <si>
-    <t>Gusto ko sana mag-resign pero may bond daw ako.</t>
-  </si>
-  <si>
-    <t>My boss is forcing me to sign a document I don't understand.</t>
-  </si>
-  <si>
-    <t>Is it true na bawal na ang placement fee sa domestic helpers?</t>
-  </si>
-  <si>
-    <t>Paano kung nag-expire na yung visa ko while waiting for the new contract?</t>
-  </si>
-  <si>
-    <t>Sinasaktan ako ng employer ko physically, saan ako tatakbo?</t>
-  </si>
-  <si>
-    <t>Paki-explain naman po yung One Month Notice rule.</t>
-  </si>
-  <si>
-    <t>Pwede ba ako mag-part time habang day off ko to earn extra?</t>
+    <t>i want to resign na sana, pero tied to bond daw ako .</t>
+  </si>
+  <si>
+    <t>Fino-force ako ng boss ko to sign a document na hindi ko gets</t>
+  </si>
+  <si>
+    <t>Is it true na bawal na ang placement fee for the domestic helpers?</t>
+  </si>
+  <si>
+    <t>what if nag-expire na yung visa ko while waiting for the new contract?</t>
+  </si>
+  <si>
+    <t>Sinasaktan ako ng employer ko physically, help me where can i complain this</t>
+  </si>
+  <si>
+    <t>pleae explain naman po yung One Month Notice rule para maintindihan ko po.</t>
+  </si>
+  <si>
+    <t>possible po ba ako mag-part time habang day off ko to earn extra?</t>
   </si>
   <si>
     <t>Kinancel nila visa ko without informing me, legal ba yun?</t>
   </si>
   <si>
-    <t>Ano gagawin ko, ayaw ako bigyan ng release letter?</t>
-  </si>
-  <si>
-    <t>Pwede ba ako mag-complain anonymously sa DOLE?</t>
-  </si>
-  <si>
-    <t>Yung sahod ko laging delayed, pwede ba ground for termination yun?</t>
+    <t>what to do po, ayaw ako bigyan ng release letter?</t>
+  </si>
+  <si>
+    <t>how can i complain anonymously sa DOLE, nahihirapan na po kasi ako sa sitwasyon ko?</t>
+  </si>
+  <si>
+    <t>my salary is delayed, ano po ang dapat ko gawin? they refuse to talk to me.</t>
   </si>
   <si>
     <t>Ask ko lang if covered ng insurance kapag na-accident sa work?</t>
@@ -312,40 +312,40 @@
     <t>Yung amo ko, he kicked me out of the house kagabi.</t>
   </si>
   <si>
-    <t>Legal ba na 24 hours naka-monitor sa CCTV sa kwarto ko?</t>
-  </si>
-  <si>
-    <t>Kailangan ba dumaan sa agency kapag direct hire?</t>
-  </si>
-  <si>
-    <t>Paano mag-claim ng OWWA benefits if member ako?</t>
-  </si>
-  <si>
-    <t>Ano ang requirements for Balik Manggagawa?</t>
-  </si>
-  <si>
-    <t>Hold departure order daw ako, paano ko malalaman?</t>
-  </si>
-  <si>
-    <t>Pwede ba mag-file ng adultery case ang asawa ko kahit nasa abroad ako?</t>
-  </si>
-  <si>
-    <t>Saan pwede mag-report ng abusive agency?</t>
-  </si>
-  <si>
-    <t>Kung ma-terminate ako, sagot ba nila ticket ko pauwi?</t>
-  </si>
-  <si>
-    <t>Valid ba yung contract if walang pirma ng POEA?</t>
-  </si>
-  <si>
-    <t>Hinaharang ako ng immigration, ano ang gagawin ko?</t>
-  </si>
-  <si>
-    <t>Puno na yung passport pages ko, pwede ba mag-renew sa consulate?</t>
-  </si>
-  <si>
-    <t>My employer didn't pay my MPF, can I report?</t>
+    <t>Legal ba na 24 hours naka-monitor ang CCTV sa room where i reside?</t>
+  </si>
+  <si>
+    <t>do i need ba na dumaan sa agency kapag direct hire?</t>
+  </si>
+  <si>
+    <t>Paano mag-claim ng OWWA benefits if i am a member?</t>
+  </si>
+  <si>
+    <t>Ano ang requirements for Balik Manggagawa please elaborate po?</t>
+  </si>
+  <si>
+    <t>Hold departure order daw ako, paano ko malalaman and what should i do?</t>
+  </si>
+  <si>
+    <t>Possible ba mag-file ng adultery case ang husband ko kahit nasa abroad ako?</t>
+  </si>
+  <si>
+    <t>where can i report abuse anong abusive agency po kaya ako mag susumbong?</t>
+  </si>
+  <si>
+    <t>Kung ma-terminate ako, will they shoulder the expense of my ticket ko pauwi?</t>
+  </si>
+  <si>
+    <t>Valid ba yung contract if no signature from POEA pero present po ang DMW signature?</t>
+  </si>
+  <si>
+    <t>Hinaharang ako ng immigration, what should i do po i am worried?</t>
+  </si>
+  <si>
+    <t>Puno na yung passport pages ko, possible po bamag-renew in the consulate?</t>
+  </si>
+  <si>
+    <t>My employer didn't pay my MPF, pano ko po kaya ito isusumbong</t>
   </si>
   <si>
     <t>我想問下如果我老細唔比通知期就炒我，合唔合法？</t>
@@ -498,6 +498,357 @@
     <t>哪裡可以找到免費法律諮詢？</t>
   </si>
   <si>
+    <t>我平時除咗做家務，老細仲日日叫我落去佢間茶餐廳幫手洗碗，咁樣係咪做緊黑工？</t>
+  </si>
+  <si>
+    <t>老板没给足加班费，我该怎么投诉？</t>
+  </si>
+  <si>
+    <t>Chinese</t>
+  </si>
+  <si>
+    <t>我的工资已经拖欠两个月了。</t>
+  </si>
+  <si>
+    <t>雇主可以因为我打破东西就扣我工资吗？</t>
+  </si>
+  <si>
+    <t>如果我还没做满一年，辞职有年终奖吗？</t>
+  </si>
+  <si>
+    <t>为什么我的工资单里扣了这么多中介费？</t>
+  </si>
+  <si>
+    <t>合同里说有伙食津贴，但老板一直没给。</t>
+  </si>
+  <si>
+    <t>我生病请假，雇主说要扣除当天的全薪。</t>
+  </si>
+  <si>
+    <t>遣散费应该怎么计算？</t>
+  </si>
+  <si>
+    <t>老板说没钱发工资，让我等下个月，这合法吗？</t>
+  </si>
+  <si>
+    <t>如果我被即时解雇，能拿到代通知金吗？</t>
+  </si>
+  <si>
+    <t>我每天工作超过16个小时，完全没有休息时间。</t>
+  </si>
+  <si>
+    <t>雇主强迫我在法定假日工作，还不给补假。</t>
+  </si>
+  <si>
+    <t>每周一天的休息日，雇主不准我出门。</t>
+  </si>
+  <si>
+    <t>我可以把今年的年假累积到明年吗？</t>
+  </si>
+  <si>
+    <t>老板要求我随叫随到，这算不算工作时间？</t>
+  </si>
+  <si>
+    <t>如果我在休息日加班，工资该怎么算？</t>
+  </si>
+  <si>
+    <t>我想请事假回国参加葬礼，雇主不批怎么办？</t>
+  </si>
+  <si>
+    <t>劳动法规定每天最少必须休息几个小时？</t>
+  </si>
+  <si>
+    <t>我的合同快到期了，续约的流程是什么？</t>
+  </si>
+  <si>
+    <t>雇主把我的护照没收了，不肯还给我。</t>
+  </si>
+  <si>
+    <t>如果我中途辞职，需要赔偿老板多少钱？</t>
+  </si>
+  <si>
+    <t>签证还有两天就过期了，我会被遣返吗？</t>
+  </si>
+  <si>
+    <t>雇主去世了，我的工作合同还有效吗？</t>
+  </si>
+  <si>
+    <t>我可以在试用期内不需要通知期就离职吗？</t>
+  </si>
+  <si>
+    <t>现在的雇主要移民了，我可以转聘给新雇主吗？</t>
+  </si>
+  <si>
+    <t>合同上写的地址和实际工作的地址不一样，有问题吗？</t>
+  </si>
+  <si>
+    <t>老板不给我提供床位，让我睡在客厅地板上。</t>
+  </si>
+  <si>
+    <t>宿舍环境非常恶劣，到处都是蟑螂和老鼠。</t>
+  </si>
+  <si>
+    <t>如果我被误控偷窃并被警方扣留，中介有义务帮我吗？</t>
+  </si>
+  <si>
+    <t>我在工作时从高处摔下来受伤了，老板不肯出医药费。</t>
+  </si>
+  <si>
+    <t>老板没帮我买工伤保险，我现在受伤了怎么办？</t>
+  </si>
+  <si>
+    <t>他们不让我吃饱饭，这算不算虐待？</t>
+  </si>
+  <si>
+    <t>如果老板的公司破产了，我的欠薪是由政府代付吗？</t>
+  </si>
+  <si>
+    <t>老板总是对我大声辱骂，甚至动手打我。</t>
+  </si>
+  <si>
+    <t>雇主威胁我要报警指控我偷东西，但我没做过。</t>
+  </si>
+  <si>
+    <t>我怀孕了，老板知道后马上说要开除我。</t>
+  </si>
+  <si>
+    <t>老板不准我参加周日的宗教活动。</t>
+  </si>
+  <si>
+    <t>老板强迫我签署一份我不理解的文件，该怎么办？</t>
+  </si>
+  <si>
+    <t>如果我丢失了身份证，在补办期间工作是合法的吗？</t>
+  </si>
+  <si>
+    <t>雇主强迫我去做合同以外的危险工作。</t>
+  </si>
+  <si>
+    <t>哪里可以找到免费的法律咨询服务？</t>
+  </si>
+  <si>
+    <t>劳工处的投诉电话是多少？</t>
+  </si>
+  <si>
+    <t>离职后的回程机票应该是雇主买吗？</t>
+  </si>
+  <si>
+    <t>我怀疑老板从我的工资里偷扣了强积金的份额。</t>
+  </si>
+  <si>
+    <t>老板要求我去他的餐厅帮手，但我只是家庭佣工，这合法吗？</t>
+  </si>
+  <si>
+    <t>菲律宾领事馆能帮我处理劳资纠纷吗？</t>
+  </si>
+  <si>
+    <t>我想终止合约，需要提前多久给书面通知？</t>
+  </si>
+  <si>
+    <t>强积金或社保应该由谁缴纳？</t>
+  </si>
+  <si>
+    <t>如果我决定回国，我的签证记录会有影响吗？</t>
+  </si>
+  <si>
+    <t>老板要求我到他朋友家帮忙打扫，这违反劳动法吗？</t>
+  </si>
+  <si>
+    <t>Attorney, my employer confiscated my passport on my very first day, is this legal?</t>
+  </si>
+  <si>
+    <t>English</t>
+  </si>
+  <si>
+    <t>I haven't been allowed to take a single day off by my employer for three months now, what should I do?</t>
+  </si>
+  <si>
+    <t>Do I have the right to file a formal complaint if the patient I am caring for physically hurts me?</t>
+  </si>
+  <si>
+    <t>I want to go back to the Philippines, but my employer refuses to give me my return ticket.</t>
+  </si>
+  <si>
+    <t>The agency forced me to sign a new contract here abroad that has a much lower salary than what we agreed upon in Manila.</t>
+  </si>
+  <si>
+    <t>My employer is deducting the cost of my food and basic toiletries from my monthly salary without my consent, is that allowed?</t>
+  </si>
+  <si>
+    <t>I am being forced to work for my employer's relatives in a different house, which is clearly not part of my employment contract.</t>
+  </si>
+  <si>
+    <t>Can I terminate my contract early and demand repatriation because my employer constantly verbally abuses me?</t>
+  </si>
+  <si>
+    <t>I have been working here for two years, but my employer still hasn't paid my salary for the last three months.</t>
+  </si>
+  <si>
+    <t>My Philippine agency ignores all my messages asking for help with my abusive employer; can I hold them liable?</t>
+  </si>
+  <si>
+    <t>Is it a labor violation for my employer to lock me from the outside whenever they leave the house?</t>
+  </si>
+  <si>
+    <t>I am extremely sick, but my employer refuses to take me to the hospital or even buy me basic medicine.</t>
+  </si>
+  <si>
+    <t>My employer forces me to work 16 hours a day with only short 10-minute breaks for meals.</t>
+  </si>
+  <si>
+    <t>I want to resign due to severe homesickness, but my employer is asking me to pay them a huge penalty fee before they let me go.</t>
+  </si>
+  <si>
+    <t>The recruitment agency collected an exorbitant placement fee from me, and now I am drowning in debt. How can I report them to the DMW?</t>
+  </si>
+  <si>
+    <t>Can my employer legally withhold my salary until my contract ends to ensure I don't run away?</t>
+  </si>
+  <si>
+    <t>How do I legally process a claim for unpaid wages and illegal dismissal against my former employer if I have already returned to the Philippines?</t>
+  </si>
+  <si>
+    <t>I caught my employer's husband secretly taking photos of me while I was in my room; how can I report this safely without getting deported?</t>
+  </si>
+  <si>
+    <t>I am not provided with proper sleeping quarters and I am forced to sleep on the cold kitchen floor.</t>
+  </si>
+  <si>
+    <t>My contract has officially expired, but my employer refuses to process my exit visa so I can go home.</t>
+  </si>
+  <si>
+    <t>I was deployed as a domestic helper, but upon arrival, I was illegally forced to work in a commercial restaurant owned by my sponsor.</t>
+  </si>
+  <si>
+    <t>If I break my contract due to a family emergency back home, do I still need to reimburse my employer's deployment expenses?</t>
+  </si>
+  <si>
+    <t>My employer only feeds me leftover food once a day; is this enough grounds for immediate repatriation under DMW rules?</t>
+  </si>
+  <si>
+    <t>I just found out I am pregnant, and my employer is threatening to deport me immediately without paying my final salary.</t>
+  </si>
+  <si>
+    <t>The foreign agency in my host country is threatening to hand me over to the police if I complain about my harsh working conditions.</t>
+  </si>
+  <si>
+    <t>Are OFWs entitled to overtime pay if they are made to work during public holidays in the host country?</t>
+  </si>
+  <si>
+    <t>My employer refuses to give me my end-of-service benefits after successfully completing my two-year contract.</t>
+  </si>
+  <si>
+    <t>I suffered a work-related injury, but my employer refuses to pay for my medical bills or give me time to recover.</t>
+  </si>
+  <si>
+    <t>Is it legal for my local recruitment agency to automatically deduct a portion of my monthly salary as a continuous "service fee"?</t>
+  </si>
+  <si>
+    <t>Attorney, my employer is constantly threatening to falsely accuse me of theft if I make a minor mistake in my chores.</t>
+  </si>
+  <si>
+    <t>I want to transfer to a different employer because of physical abuse, but my current sponsor refuses to give me a release paper.</t>
+  </si>
+  <si>
+    <t>Can my employer force me to clean their cars and their neighbors' cars without extra compensation?</t>
+  </si>
+  <si>
+    <t>My employer forces me to surrender my ATM bank card and PIN where my monthly salary is supposedly deposited.</t>
+  </si>
+  <si>
+    <t>The agency recruiter in the Philippines promised me a $600 salary, but the contract they gave me at the airport only stated $400.</t>
+  </si>
+  <si>
+    <t>I want to seek refuge at the Philippine embassy, but I am afraid my employer will file false absconding charges against me to get me arrested.</t>
+  </si>
+  <si>
+    <t>I was promised free accommodation in my original contract, but my employer is now charging me monthly rent.</t>
+  </si>
+  <si>
+    <t>My employer confiscated my mobile phone and only allows me to call my family once a month for exactly five minutes.</t>
+  </si>
+  <si>
+    <t>I just discovered that the visa issued to me is a tourist visa instead of a legal working visa; what are my options to legalize my stay or go home safely?</t>
+  </si>
+  <si>
+    <t>The foreign placement agency sold me to another employer without my knowledge and consent; is this considered human trafficking?</t>
+  </si>
+  <si>
+    <t>I am experiencing severe depression due to isolation; can the DMW help me get repatriated on medical grounds even if my contract isn't finished?</t>
+  </si>
+  <si>
+    <t>My employer strictly forbids me from practicing my religion or praying inside my own room.</t>
+  </si>
+  <si>
+    <t>I have been working under a renewed contract, but I found out it was not verified by the Migrant Workers Office (MWO). Will this affect my OFW benefits?</t>
+  </si>
+  <si>
+    <t>My employer passed away, and their family immediately kicked me out of the house without giving me my unpaid wages for the last two months.</t>
+  </si>
+  <si>
+    <t>Is it a violation of my privacy rights if my employer installs CCTV cameras inside my private bedroom and bathroom?</t>
+  </si>
+  <si>
+    <t>The local agency told me that I have to pay for my own return ticket even though I finished my contract successfully. Is that true?</t>
+  </si>
+  <si>
+    <t>My employer physically assaulted me, but the local police dismissed my complaint because my employer is an influential local citizen. Where can I seek legal help?</t>
+  </si>
+  <si>
+    <t>I am constantly being denied my weekly legal rest day, and if I complain, my employer cuts my internet access as punishment.</t>
+  </si>
+  <si>
+    <t>I signed a contract as a registered nurse, but my employer assigned me as a personal caregiver doing heavy household chores and cleaning.</t>
+  </si>
+  <si>
+    <t>Can I file a case against my Philippine agency for deploying me to an employer with a known public history of abusing domestic workers?</t>
+  </si>
+  <si>
+    <t>My employer is withholding my final pay, claiming that I broke expensive household items, which is entirely false.</t>
+  </si>
+  <si>
+    <t>likert_natural(ScaleOf1to5)</t>
+  </si>
+  <si>
+    <t>suggested_prompt(spoken)</t>
+  </si>
+  <si>
+    <t>The employer's failure to provide notice period prior to termination is unlawful.</t>
+  </si>
+  <si>
+    <t>勞工處個電話係咩？我想問下工傷賠償。</t>
+  </si>
+  <si>
+    <t>欠債會唔會影響我嘅申請簽證？</t>
+  </si>
+  <si>
+    <t>僱主過左世，我份合約仲有冇效？</t>
+  </si>
+  <si>
+    <t>簽咗約但我後悔，可唔可以取消？</t>
+  </si>
+  <si>
+    <t>佢地係廁所裝咗CCTV，我好驚。</t>
+  </si>
+  <si>
+    <t>被人無理解僱，有無得賠償？</t>
+  </si>
+  <si>
+    <t>簽證被人拒絕，我要幾時離境？</t>
+  </si>
+  <si>
+    <t>有勞資糾紛嘅話，係咪要去領事館搞掂？</t>
+  </si>
+  <si>
+    <t>如果我受左傷，係咪工傷？</t>
+  </si>
+  <si>
+    <t>我老細移民，我係咪要跟埋一齊去？</t>
+  </si>
+  <si>
+    <t>邊度可以搵到免費法律諮詢？</t>
+  </si>
+  <si>
     <t>我啱啱發現有咗BB，老細知道之後即刻話要炒我，香港法例係咪容許咁樣？</t>
   </si>
   <si>
@@ -547,51 +898,6 @@
   </si>
   <si>
     <t>婆婆（受照顧者）過身，佢個仔話合約即刻完，要我聽日就買機票返菲律賓，咁我啲遣散費點計？</t>
-  </si>
-  <si>
-    <t>我平時除咗做家務，老細仲日日叫我落去佢間茶餐廳幫手洗碗，咁樣係咪做緊黑工？</t>
-  </si>
-  <si>
-    <t>likert_natural(ScaleOf1to5)</t>
-  </si>
-  <si>
-    <t>suggested_prompt(spoken)</t>
-  </si>
-  <si>
-    <t>The employer's failure to provide notice period prior to termination is unlawful.</t>
-  </si>
-  <si>
-    <t>勞工處個電話係咩？我想問下工傷賠償。</t>
-  </si>
-  <si>
-    <t>欠債會唔會影響我嘅申請簽證？</t>
-  </si>
-  <si>
-    <t>僱主過左世，我份合約仲有冇效？</t>
-  </si>
-  <si>
-    <t>簽咗約但我後悔，可唔可以取消？</t>
-  </si>
-  <si>
-    <t>佢地係廁所裝咗CCTV，我好驚。</t>
-  </si>
-  <si>
-    <t>被人無理解僱，有無得賠償？</t>
-  </si>
-  <si>
-    <t>簽證被人拒絕，我要幾時離境？</t>
-  </si>
-  <si>
-    <t>有勞資糾紛嘅話，係咪要去領事館搞掂？</t>
-  </si>
-  <si>
-    <t>如果我受左傷，係咪工傷？</t>
-  </si>
-  <si>
-    <t>我老細移民，我係咪要跟埋一齊去？</t>
-  </si>
-  <si>
-    <t>邊度可以搵到免費法律諮詢？</t>
   </si>
 </sst>
 </file>
@@ -599,10 +905,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
   <numFmts count="4">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="179" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -965,12 +1271,42 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="11">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -1077,16 +1413,16 @@
     <xf numFmtId="176" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="177" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="178" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="179" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1095,7 +1431,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1107,34 +1443,34 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1219,11 +1555,17 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1238,7 +1580,7 @@
     <cellStyle name="Note" xfId="8" builtinId="10"/>
     <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
     <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
     <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
     <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
     <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
@@ -1700,13 +2042,13 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:D168"/>
-  <sheetFormatPr defaultColWidth="12.6296296296296" defaultRowHeight="15.75" customHeight="1" outlineLevelCol="3"/>
+  <dimension ref="A1:D251"/>
+  <sheetFormatPr defaultColWidth="12.6285714285714" defaultRowHeight="15.75" customHeight="1" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="1" width="72" customWidth="1"/>
-    <col min="2" max="2" width="19.6296296296296" customWidth="1"/>
+    <col min="2" max="2" width="19.6285714285714" customWidth="1"/>
     <col min="3" max="3" width="37" customWidth="1"/>
-    <col min="4" max="4" width="36.75" customWidth="1"/>
+    <col min="4" max="4" width="36.752380952381" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" customHeight="1" spans="1:4">
@@ -1723,1340 +2065,2004 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" customHeight="1" spans="1:4">
-      <c r="A2" s="1" t="s">
+    <row r="2" customHeight="1" spans="1:2">
+      <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" customHeight="1" spans="1:4">
-      <c r="A3" s="1" t="s">
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" customHeight="1" spans="1:2">
+      <c r="A3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" customHeight="1" spans="1:4">
-      <c r="A4" s="1" t="s">
+      <c r="B3" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" customHeight="1" spans="1:2">
+      <c r="A4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" customHeight="1" spans="1:4">
-      <c r="A5" s="1" t="s">
+      <c r="B4" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" customHeight="1" spans="1:2">
+      <c r="A5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" customHeight="1" spans="1:4">
-      <c r="A6" s="1" t="s">
+      <c r="B5" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" customHeight="1" spans="1:2">
+      <c r="A6" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" customHeight="1" spans="1:4">
-      <c r="A7" s="1" t="s">
+      <c r="B6" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" customHeight="1" spans="1:2">
+      <c r="A7" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" customHeight="1" spans="1:4">
-      <c r="A8" s="1" t="s">
+      <c r="B7" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" customHeight="1" spans="1:2">
+      <c r="A8" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" customHeight="1" spans="1:4">
-      <c r="A9" s="1" t="s">
+      <c r="B8" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" customHeight="1" spans="1:2">
+      <c r="A9" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10" customHeight="1" spans="1:4">
-      <c r="A10" s="1" t="s">
+      <c r="B9" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" customHeight="1" spans="1:2">
+      <c r="A10" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11" customHeight="1" spans="1:4">
-      <c r="A11" s="1" t="s">
+      <c r="B10" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" customHeight="1" spans="1:2">
+      <c r="A11" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="12" customHeight="1" spans="1:4">
-      <c r="A12" s="1" t="s">
+      <c r="B11" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" customHeight="1" spans="1:2">
+      <c r="A12" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="13" customHeight="1" spans="1:4">
-      <c r="A13" s="1" t="s">
+      <c r="B12" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" customHeight="1" spans="1:2">
+      <c r="A13" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="14" customHeight="1" spans="1:4">
-      <c r="A14" s="1" t="s">
+      <c r="B13" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" customHeight="1" spans="1:2">
+      <c r="A14" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="15" customHeight="1" spans="1:4">
-      <c r="A15" s="1" t="s">
+      <c r="B14" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" customHeight="1" spans="1:2">
+      <c r="A15" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="16" customHeight="1" spans="1:4">
-      <c r="A16" s="1" t="s">
+      <c r="B15" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" customHeight="1" spans="1:2">
+      <c r="A16" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="17" customHeight="1" spans="1:2">
-      <c r="A17" s="1" t="s">
+      <c r="A17" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="18" customHeight="1" spans="1:2">
-      <c r="A18" s="1" t="s">
+      <c r="A18" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="19" customHeight="1" spans="1:2">
-      <c r="A19" s="1" t="s">
+      <c r="A19" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="20" customHeight="1" spans="1:2">
-      <c r="A20" s="1" t="s">
+      <c r="A20" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="21" customHeight="1" spans="1:2">
-      <c r="A21" s="1" t="s">
+      <c r="A21" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="22" customHeight="1" spans="1:2">
-      <c r="A22" s="1" t="s">
+      <c r="A22" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B22" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="23" customHeight="1" spans="1:2">
-      <c r="A23" s="1" t="s">
+      <c r="A23" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="24" customHeight="1" spans="1:2">
-      <c r="A24" s="1" t="s">
+      <c r="A24" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B24" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="25" customHeight="1" spans="1:2">
-      <c r="A25" s="1" t="s">
+      <c r="A25" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="B25" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="26" customHeight="1" spans="1:2">
-      <c r="A26" s="1" t="s">
+      <c r="A26" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B26" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="27" customHeight="1" spans="1:2">
-      <c r="A27" s="1" t="s">
+      <c r="A27" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B27" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="28" customHeight="1" spans="1:2">
-      <c r="A28" s="1" t="s">
+      <c r="A28" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B28" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="29" customHeight="1" spans="1:2">
-      <c r="A29" s="1" t="s">
+      <c r="A29" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B29" s="1" t="s">
+      <c r="B29" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="30" customHeight="1" spans="1:2">
-      <c r="A30" s="1" t="s">
+      <c r="A30" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B30" s="1" t="s">
+      <c r="B30" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="31" customHeight="1" spans="1:2">
-      <c r="A31" s="1" t="s">
+      <c r="A31" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="B31" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="32" customHeight="1" spans="1:2">
-      <c r="A32" s="1" t="s">
+      <c r="A32" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="B32" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="33" customHeight="1" spans="1:2">
-      <c r="A33" s="1" t="s">
+      <c r="A33" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="B33" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="34" customHeight="1" spans="1:2">
-      <c r="A34" s="1" t="s">
+      <c r="A34" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="B34" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="35" customHeight="1" spans="1:2">
-      <c r="A35" s="1" t="s">
+      <c r="A35" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="B35" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="36" customHeight="1" spans="1:2">
-      <c r="A36" s="1" t="s">
+      <c r="A36" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="B36" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="37" customHeight="1" spans="1:2">
-      <c r="A37" s="1" t="s">
+      <c r="A37" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="B37" s="1" t="s">
+      <c r="B37" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="38" customHeight="1" spans="1:2">
-      <c r="A38" s="1" t="s">
+      <c r="A38" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="B38" s="1" t="s">
+      <c r="B38" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="39" customHeight="1" spans="1:2">
-      <c r="A39" s="1" t="s">
+      <c r="A39" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B39" s="1" t="s">
+      <c r="B39" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="40" customHeight="1" spans="1:2">
-      <c r="A40" s="1" t="s">
+      <c r="A40" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="B40" s="1" t="s">
+      <c r="B40" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="41" customHeight="1" spans="1:2">
-      <c r="A41" s="1" t="s">
+      <c r="A41" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="B41" s="1" t="s">
+      <c r="B41" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="42" customHeight="1" spans="1:2">
-      <c r="A42" s="1" t="s">
+      <c r="A42" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="B42" s="1" t="s">
+      <c r="B42" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="43" customHeight="1" spans="1:2">
-      <c r="A43" s="1" t="s">
+      <c r="A43" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B43" s="1" t="s">
+      <c r="B43" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="44" customHeight="1" spans="1:2">
-      <c r="A44" s="1" t="s">
+      <c r="A44" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="B44" s="1" t="s">
+      <c r="B44" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="45" customHeight="1" spans="1:2">
-      <c r="A45" s="1" t="s">
+      <c r="A45" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B45" s="1" t="s">
+      <c r="B45" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="46" customHeight="1" spans="1:2">
-      <c r="A46" s="1" t="s">
+      <c r="A46" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="B46" s="1" t="s">
+      <c r="B46" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="47" customHeight="1" spans="1:2">
-      <c r="A47" s="1" t="s">
+      <c r="A47" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="B47" s="1" t="s">
+      <c r="B47" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="48" customHeight="1" spans="1:2">
-      <c r="A48" s="1" t="s">
+      <c r="A48" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B48" s="1" t="s">
+      <c r="B48" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="49" customHeight="1" spans="1:2">
-      <c r="A49" s="1" t="s">
+      <c r="A49" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="B49" s="1" t="s">
+      <c r="B49" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="50" customHeight="1" spans="1:2">
-      <c r="A50" s="1" t="s">
+      <c r="A50" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B50" s="1" t="s">
+      <c r="B50" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="51" customHeight="1" spans="1:2">
-      <c r="A51" s="1" t="s">
+      <c r="A51" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B51" s="1" t="s">
+      <c r="B51" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="52" customHeight="1" spans="1:2">
-      <c r="A52" s="1" t="s">
+      <c r="A52" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="B52" s="1" t="s">
+      <c r="B52" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="53" customHeight="1" spans="1:2">
-      <c r="A53" s="1" t="s">
+      <c r="A53" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B53" s="1" t="s">
+      <c r="B53" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="54" customHeight="1" spans="1:2">
-      <c r="A54" s="1" t="s">
+      <c r="A54" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="B54" s="1" t="s">
+      <c r="B54" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="55" customHeight="1" spans="1:2">
-      <c r="A55" s="1" t="s">
+      <c r="A55" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="B55" s="1" t="s">
+      <c r="B55" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="56" customHeight="1" spans="1:2">
-      <c r="A56" s="1" t="s">
+      <c r="A56" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B56" s="1" t="s">
+      <c r="B56" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="57" customHeight="1" spans="1:2">
-      <c r="A57" s="1" t="s">
+      <c r="A57" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="B57" s="1" t="s">
+      <c r="B57" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="58" customHeight="1" spans="1:2">
-      <c r="A58" s="1" t="s">
+      <c r="A58" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B58" s="1" t="s">
+      <c r="B58" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="59" customHeight="1" spans="1:2">
-      <c r="A59" s="1" t="s">
+      <c r="A59" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="B59" s="1" t="s">
+      <c r="B59" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="60" customHeight="1" spans="1:2">
-      <c r="A60" s="1" t="s">
+      <c r="A60" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="B60" s="1" t="s">
+      <c r="B60" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="61" customHeight="1" spans="1:2">
-      <c r="A61" s="1" t="s">
+      <c r="A61" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="B61" s="1" t="s">
+      <c r="B61" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="62" customHeight="1" spans="1:2">
-      <c r="A62" s="1" t="s">
+      <c r="A62" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="B62" s="1" t="s">
+      <c r="B62" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="63" customHeight="1" spans="1:2">
-      <c r="A63" s="1" t="s">
+      <c r="A63" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="B63" s="1" t="s">
+      <c r="B63" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="64" customHeight="1" spans="1:2">
-      <c r="A64" s="1" t="s">
+      <c r="A64" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B64" s="1" t="s">
+      <c r="B64" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="65" customHeight="1" spans="1:2">
-      <c r="A65" s="1" t="s">
+      <c r="A65" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B65" s="1" t="s">
+      <c r="B65" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="66" customHeight="1" spans="1:2">
-      <c r="A66" s="1" t="s">
+      <c r="A66" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="B66" s="1" t="s">
+      <c r="B66" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="67" customHeight="1" spans="1:2">
-      <c r="A67" s="1" t="s">
+      <c r="A67" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="B67" s="1" t="s">
+      <c r="B67" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="68" customHeight="1" spans="1:2">
-      <c r="A68" s="1" t="s">
+      <c r="A68" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="B68" s="1" t="s">
+      <c r="B68" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="69" customHeight="1" spans="1:2">
-      <c r="A69" s="1" t="s">
+      <c r="A69" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="B69" s="1" t="s">
+      <c r="B69" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="70" customHeight="1" spans="1:2">
-      <c r="A70" s="1" t="s">
+      <c r="A70" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="B70" s="1" t="s">
+      <c r="B70" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="71" customHeight="1" spans="1:2">
-      <c r="A71" s="1" t="s">
+      <c r="A71" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="B71" s="1" t="s">
+      <c r="B71" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="72" customHeight="1" spans="1:2">
-      <c r="A72" s="1" t="s">
+      <c r="A72" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="B72" s="1" t="s">
+      <c r="B72" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="73" customHeight="1" spans="1:2">
-      <c r="A73" s="1" t="s">
+      <c r="A73" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="B73" s="1" t="s">
+      <c r="B73" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="74" customHeight="1" spans="1:2">
-      <c r="A74" s="1" t="s">
+      <c r="A74" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="B74" s="1" t="s">
+      <c r="B74" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="75" customHeight="1" spans="1:2">
-      <c r="A75" s="1" t="s">
+      <c r="A75" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="B75" s="1" t="s">
+      <c r="B75" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="76" customHeight="1" spans="1:2">
-      <c r="A76" s="1" t="s">
+      <c r="A76" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="B76" s="1" t="s">
+      <c r="B76" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="77" customHeight="1" spans="1:2">
-      <c r="A77" s="1" t="s">
+      <c r="A77" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="B77" s="1" t="s">
+      <c r="B77" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="78" customHeight="1" spans="1:2">
-      <c r="A78" s="1" t="s">
+      <c r="A78" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="B78" s="1" t="s">
+      <c r="B78" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="79" customHeight="1" spans="1:2">
-      <c r="A79" s="1" t="s">
+      <c r="A79" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="B79" s="1" t="s">
+      <c r="B79" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="80" customHeight="1" spans="1:2">
-      <c r="A80" s="1" t="s">
+      <c r="A80" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="B80" s="1" t="s">
+      <c r="B80" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="81" customHeight="1" spans="1:2">
-      <c r="A81" s="1" t="s">
+      <c r="A81" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="B81" s="1" t="s">
+      <c r="B81" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="82" customHeight="1" spans="1:2">
-      <c r="A82" s="1" t="s">
+      <c r="A82" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="B82" s="1" t="s">
+      <c r="B82" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="83" customHeight="1" spans="1:2">
-      <c r="A83" s="1" t="s">
+      <c r="A83" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="B83" s="1" t="s">
+      <c r="B83" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="84" customHeight="1" spans="1:2">
-      <c r="A84" s="1" t="s">
+      <c r="A84" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B84" s="1" t="s">
+      <c r="B84" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="85" customHeight="1" spans="1:2">
-      <c r="A85" s="1" t="s">
+      <c r="A85" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="B85" s="1" t="s">
+      <c r="B85" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="86" customHeight="1" spans="1:2">
-      <c r="A86" s="1" t="s">
+      <c r="A86" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="B86" s="1" t="s">
+      <c r="B86" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="87" customHeight="1" spans="1:2">
-      <c r="A87" s="1" t="s">
+      <c r="A87" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="B87" s="1" t="s">
+      <c r="B87" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="88" customHeight="1" spans="1:2">
-      <c r="A88" s="1" t="s">
+      <c r="A88" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="B88" s="1" t="s">
+      <c r="B88" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="89" customHeight="1" spans="1:2">
-      <c r="A89" s="1" t="s">
+      <c r="A89" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="B89" s="1" t="s">
+      <c r="B89" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="90" customHeight="1" spans="1:2">
-      <c r="A90" s="1" t="s">
+      <c r="A90" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="B90" s="1" t="s">
+      <c r="B90" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="91" customHeight="1" spans="1:2">
-      <c r="A91" s="1" t="s">
+      <c r="A91" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="B91" s="1" t="s">
+      <c r="B91" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="92" customHeight="1" spans="1:2">
-      <c r="A92" s="1" t="s">
+      <c r="A92" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="B92" s="1" t="s">
+      <c r="B92" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="93" customHeight="1" spans="1:2">
-      <c r="A93" s="1" t="s">
+      <c r="A93" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="B93" s="1" t="s">
+      <c r="B93" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="94" customHeight="1" spans="1:2">
-      <c r="A94" s="1" t="s">
+      <c r="A94" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="B94" s="1" t="s">
+      <c r="B94" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="95" customHeight="1" spans="1:2">
-      <c r="A95" s="1" t="s">
+      <c r="A95" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="B95" s="1" t="s">
+      <c r="B95" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="96" customHeight="1" spans="1:2">
-      <c r="A96" s="1" t="s">
+      <c r="A96" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="B96" s="1" t="s">
+      <c r="B96" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="97" customHeight="1" spans="1:2">
-      <c r="A97" s="1" t="s">
+      <c r="A97" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="B97" s="1" t="s">
+      <c r="B97" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="98" customHeight="1" spans="1:2">
-      <c r="A98" s="1" t="s">
+      <c r="A98" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="B98" s="1" t="s">
+      <c r="B98" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="99" customHeight="1" spans="1:2">
-      <c r="A99" s="1" t="s">
+      <c r="A99" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="B99" s="1" t="s">
+      <c r="B99" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="100" customHeight="1" spans="1:2">
-      <c r="A100" s="1" t="s">
+      <c r="A100" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="B100" s="1" t="s">
+      <c r="B100" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="101" customHeight="1" spans="1:2">
-      <c r="A101" s="1" t="s">
+      <c r="A101" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="B101" s="1" t="s">
+      <c r="B101" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="102" customHeight="1" spans="1:2">
-      <c r="A102" s="1" t="s">
+      <c r="A102" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="B102" s="1" t="s">
+      <c r="B102" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="103" customHeight="1" spans="1:2">
-      <c r="A103" s="1" t="s">
+      <c r="A103" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="B103" s="1" t="s">
+      <c r="B103" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="104" customHeight="1" spans="1:2">
-      <c r="A104" s="1" t="s">
+      <c r="A104" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="B104" s="1" t="s">
+      <c r="B104" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="105" customHeight="1" spans="1:2">
-      <c r="A105" s="1" t="s">
+      <c r="A105" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="B105" s="1" t="s">
+      <c r="B105" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="106" customHeight="1" spans="1:2">
-      <c r="A106" s="1" t="s">
+      <c r="A106" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="B106" s="1" t="s">
+      <c r="B106" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="107" customHeight="1" spans="1:2">
-      <c r="A107" s="1" t="s">
+      <c r="A107" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="B107" s="1" t="s">
+      <c r="B107" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="108" customHeight="1" spans="1:2">
-      <c r="A108" s="1" t="s">
+      <c r="A108" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="B108" s="1" t="s">
+      <c r="B108" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="109" customHeight="1" spans="1:2">
-      <c r="A109" s="1" t="s">
+      <c r="A109" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="B109" s="1" t="s">
+      <c r="B109" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="110" customHeight="1" spans="1:2">
-      <c r="A110" s="1" t="s">
+      <c r="A110" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="B110" s="1" t="s">
+      <c r="B110" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="111" customHeight="1" spans="1:2">
-      <c r="A111" s="1" t="s">
+      <c r="A111" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="B111" s="1" t="s">
+      <c r="B111" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="112" customHeight="1" spans="1:2">
-      <c r="A112" s="1" t="s">
+      <c r="A112" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="B112" s="1" t="s">
+      <c r="B112" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="113" customHeight="1" spans="1:2">
-      <c r="A113" s="1" t="s">
+      <c r="A113" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="B113" s="1" t="s">
+      <c r="B113" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="114" customHeight="1" spans="1:2">
-      <c r="A114" s="1" t="s">
+      <c r="A114" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="B114" s="1" t="s">
+      <c r="B114" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="115" customHeight="1" spans="1:2">
-      <c r="A115" s="1" t="s">
+      <c r="A115" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="B115" s="1" t="s">
+      <c r="B115" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="116" customHeight="1" spans="1:2">
-      <c r="A116" s="1" t="s">
+      <c r="A116" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="B116" s="1" t="s">
+      <c r="B116" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="117" customHeight="1" spans="1:2">
-      <c r="A117" s="1" t="s">
+      <c r="A117" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="B117" s="1" t="s">
+      <c r="B117" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="118" customHeight="1" spans="1:2">
-      <c r="A118" s="1" t="s">
+      <c r="A118" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="B118" s="1" t="s">
+      <c r="B118" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="119" customHeight="1" spans="1:2">
-      <c r="A119" s="1" t="s">
+      <c r="A119" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="B119" s="1" t="s">
+      <c r="B119" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="120" customHeight="1" spans="1:2">
-      <c r="A120" s="1" t="s">
+      <c r="A120" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="B120" s="1" t="s">
+      <c r="B120" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="121" customHeight="1" spans="1:2">
-      <c r="A121" s="1" t="s">
+      <c r="A121" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="B121" s="1" t="s">
+      <c r="B121" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="122" customHeight="1" spans="1:2">
-      <c r="A122" s="1" t="s">
+      <c r="A122" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="B122" s="1" t="s">
+      <c r="B122" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="123" customHeight="1" spans="1:2">
-      <c r="A123" s="1" t="s">
+      <c r="A123" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="B123" s="1" t="s">
+      <c r="B123" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="124" customHeight="1" spans="1:2">
-      <c r="A124" s="1" t="s">
+      <c r="A124" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="B124" s="1" t="s">
+      <c r="B124" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="125" customHeight="1" spans="1:2">
-      <c r="A125" s="1" t="s">
+      <c r="A125" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="B125" s="1" t="s">
+      <c r="B125" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="126" customHeight="1" spans="1:2">
-      <c r="A126" s="1" t="s">
+      <c r="A126" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="B126" s="1" t="s">
+      <c r="B126" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="127" customHeight="1" spans="1:2">
-      <c r="A127" s="1" t="s">
+      <c r="A127" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="B127" s="1" t="s">
+      <c r="B127" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="128" customHeight="1" spans="1:2">
-      <c r="A128" s="1" t="s">
+      <c r="A128" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="B128" s="1" t="s">
+      <c r="B128" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="129" customHeight="1" spans="1:2">
-      <c r="A129" s="1" t="s">
+      <c r="A129" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="B129" s="1" t="s">
+      <c r="B129" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="130" customHeight="1" spans="1:2">
-      <c r="A130" s="1" t="s">
+      <c r="A130" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="B130" s="1" t="s">
+      <c r="B130" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="131" customHeight="1" spans="1:2">
-      <c r="A131" s="1" t="s">
+      <c r="A131" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="B131" s="1" t="s">
+      <c r="B131" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="132" customHeight="1" spans="1:2">
-      <c r="A132" s="1" t="s">
+      <c r="A132" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="B132" s="1" t="s">
+      <c r="B132" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="133" customHeight="1" spans="1:2">
-      <c r="A133" s="1" t="s">
+      <c r="A133" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="B133" s="1" t="s">
+      <c r="B133" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="134" customHeight="1" spans="1:2">
-      <c r="A134" s="1" t="s">
+      <c r="A134" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="B134" s="1" t="s">
+      <c r="B134" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="135" customHeight="1" spans="1:2">
-      <c r="A135" s="1" t="s">
+      <c r="A135" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="B135" s="1" t="s">
+      <c r="B135" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="136" customHeight="1" spans="1:2">
-      <c r="A136" s="1" t="s">
+      <c r="A136" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="B136" s="1" t="s">
+      <c r="B136" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="137" customHeight="1" spans="1:2">
-      <c r="A137" s="1" t="s">
+      <c r="A137" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="B137" s="1" t="s">
+      <c r="B137" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="138" customHeight="1" spans="1:2">
-      <c r="A138" s="1" t="s">
+      <c r="A138" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="B138" s="1" t="s">
+      <c r="B138" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="139" customHeight="1" spans="1:2">
-      <c r="A139" s="1" t="s">
+      <c r="A139" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="B139" s="1" t="s">
+      <c r="B139" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="140" customHeight="1" spans="1:2">
-      <c r="A140" s="1" t="s">
+      <c r="A140" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="B140" s="1" t="s">
+      <c r="B140" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="141" customHeight="1" spans="1:2">
-      <c r="A141" s="1" t="s">
+      <c r="A141" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="B141" s="1" t="s">
+      <c r="B141" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="142" customHeight="1" spans="1:2">
-      <c r="A142" s="1" t="s">
+      <c r="A142" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="B142" s="1" t="s">
+      <c r="B142" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="143" customHeight="1" spans="1:2">
-      <c r="A143" s="1" t="s">
+      <c r="A143" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="B143" s="1" t="s">
+      <c r="B143" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="144" customHeight="1" spans="1:2">
-      <c r="A144" s="1" t="s">
+      <c r="A144" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="B144" s="1" t="s">
+      <c r="B144" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="145" customHeight="1" spans="1:2">
-      <c r="A145" s="1" t="s">
+      <c r="A145" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="B145" s="1" t="s">
+      <c r="B145" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="146" customHeight="1" spans="1:2">
-      <c r="A146" s="1" t="s">
+      <c r="A146" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="B146" s="1" t="s">
+      <c r="B146" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="147" customHeight="1" spans="1:2">
-      <c r="A147" s="1" t="s">
+      <c r="A147" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="B147" s="1" t="s">
+      <c r="B147" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="148" customHeight="1" spans="1:2">
-      <c r="A148" s="1" t="s">
+      <c r="A148" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="B148" s="1" t="s">
+      <c r="B148" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="149" customHeight="1" spans="1:2">
-      <c r="A149" s="1" t="s">
+      <c r="A149" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="B149" s="1" t="s">
+      <c r="B149" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="150" customHeight="1" spans="1:2">
-      <c r="A150" s="1" t="s">
+      <c r="A150" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="B150" s="1" t="s">
+      <c r="B150" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="151" customHeight="1" spans="1:2">
-      <c r="A151" t="s">
+      <c r="A151" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="B151" s="1" t="s">
+      <c r="B151" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="152" customHeight="1" spans="1:2">
-      <c r="A152" t="s">
+      <c r="A152" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="B152" s="1" t="s">
-        <v>107</v>
+      <c r="B152" s="4" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="153" customHeight="1" spans="1:2">
-      <c r="A153" t="s">
+      <c r="A153" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B153" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="B153" s="1" t="s">
-        <v>107</v>
-      </c>
     </row>
     <row r="154" customHeight="1" spans="1:2">
-      <c r="A154" t="s">
-        <v>159</v>
-      </c>
-      <c r="B154" s="1" t="s">
-        <v>107</v>
+      <c r="A154" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="B154" s="4" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="155" customHeight="1" spans="1:2">
-      <c r="A155" t="s">
-        <v>160</v>
-      </c>
-      <c r="B155" s="1" t="s">
-        <v>107</v>
+      <c r="A155" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="B155" s="4" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="156" customHeight="1" spans="1:2">
-      <c r="A156" t="s">
-        <v>161</v>
-      </c>
-      <c r="B156" s="1" t="s">
-        <v>107</v>
+      <c r="A156" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="B156" s="4" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="157" customHeight="1" spans="1:2">
-      <c r="A157" t="s">
-        <v>162</v>
-      </c>
-      <c r="B157" s="1" t="s">
-        <v>107</v>
+      <c r="A157" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="B157" s="4" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="158" customHeight="1" spans="1:2">
-      <c r="A158" t="s">
-        <v>163</v>
-      </c>
-      <c r="B158" s="1" t="s">
-        <v>107</v>
+      <c r="A158" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="B158" s="4" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="159" customHeight="1" spans="1:2">
-      <c r="A159" t="s">
-        <v>164</v>
-      </c>
-      <c r="B159" s="1" t="s">
-        <v>107</v>
+      <c r="A159" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="B159" s="4" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="160" customHeight="1" spans="1:2">
-      <c r="A160" t="s">
-        <v>165</v>
-      </c>
-      <c r="B160" s="1" t="s">
-        <v>107</v>
+      <c r="A160" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="B160" s="4" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="161" customHeight="1" spans="1:2">
-      <c r="A161" t="s">
-        <v>166</v>
-      </c>
-      <c r="B161" s="1" t="s">
-        <v>107</v>
+      <c r="A161" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="B161" s="4" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="162" customHeight="1" spans="1:2">
-      <c r="A162" t="s">
-        <v>167</v>
-      </c>
-      <c r="B162" s="1" t="s">
-        <v>107</v>
+      <c r="A162" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="B162" s="4" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="163" customHeight="1" spans="1:2">
-      <c r="A163" t="s">
-        <v>168</v>
-      </c>
-      <c r="B163" s="1" t="s">
-        <v>107</v>
+      <c r="A163" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="B163" s="4" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="164" customHeight="1" spans="1:2">
-      <c r="A164" t="s">
-        <v>169</v>
-      </c>
-      <c r="B164" s="1" t="s">
-        <v>107</v>
+      <c r="A164" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="B164" s="4" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="165" customHeight="1" spans="1:2">
-      <c r="A165" t="s">
-        <v>170</v>
-      </c>
-      <c r="B165" s="1" t="s">
-        <v>107</v>
+      <c r="A165" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="B165" s="4" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="166" customHeight="1" spans="1:2">
-      <c r="A166" t="s">
-        <v>171</v>
-      </c>
-      <c r="B166" s="1" t="s">
-        <v>107</v>
+      <c r="A166" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="B166" s="4" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="167" customHeight="1" spans="1:2">
-      <c r="A167" t="s">
-        <v>172</v>
-      </c>
-      <c r="B167" s="1" t="s">
-        <v>107</v>
+      <c r="A167" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="B167" s="4" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="168" customHeight="1" spans="1:2">
-      <c r="A168" t="s">
-        <v>173</v>
-      </c>
-      <c r="B168" s="1" t="s">
-        <v>107</v>
+      <c r="A168" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="B168" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="169" customHeight="1" spans="1:2">
+      <c r="A169" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B169" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="170" customHeight="1" spans="1:2">
+      <c r="A170" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="B170" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="171" customHeight="1" spans="1:2">
+      <c r="A171" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="B171" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="172" customHeight="1" spans="1:2">
+      <c r="A172" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="B172" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="173" customHeight="1" spans="1:2">
+      <c r="A173" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="B173" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="174" customHeight="1" spans="1:2">
+      <c r="A174" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="B174" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="175" customHeight="1" spans="1:2">
+      <c r="A175" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="B175" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="176" customHeight="1" spans="1:2">
+      <c r="A176" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="B176" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="177" customHeight="1" spans="1:2">
+      <c r="A177" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="B177" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="178" customHeight="1" spans="1:2">
+      <c r="A178" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="B178" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="179" customHeight="1" spans="1:2">
+      <c r="A179" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="B179" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="180" customHeight="1" spans="1:2">
+      <c r="A180" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="B180" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="181" customHeight="1" spans="1:2">
+      <c r="A181" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="B181" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="182" customHeight="1" spans="1:2">
+      <c r="A182" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="B182" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="183" customHeight="1" spans="1:2">
+      <c r="A183" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="B183" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="184" customHeight="1" spans="1:2">
+      <c r="A184" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="B184" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="185" customHeight="1" spans="1:2">
+      <c r="A185" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="B185" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="186" customHeight="1" spans="1:2">
+      <c r="A186" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="B186" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="187" customHeight="1" spans="1:2">
+      <c r="A187" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="B187" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="188" customHeight="1" spans="1:2">
+      <c r="A188" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="B188" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="189" customHeight="1" spans="1:2">
+      <c r="A189" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="B189" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="190" customHeight="1" spans="1:2">
+      <c r="A190" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="B190" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="191" customHeight="1" spans="1:2">
+      <c r="A191" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="B191" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="192" customHeight="1" spans="1:2">
+      <c r="A192" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="B192" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="193" customHeight="1" spans="1:2">
+      <c r="A193" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="B193" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="194" customHeight="1" spans="1:2">
+      <c r="A194" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="B194" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="195" customHeight="1" spans="1:2">
+      <c r="A195" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="B195" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="196" customHeight="1" spans="1:2">
+      <c r="A196" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="B196" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="197" customHeight="1" spans="1:2">
+      <c r="A197" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B197" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="198" customHeight="1" spans="1:2">
+      <c r="A198" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="B198" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="199" customHeight="1" spans="1:2">
+      <c r="A199" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="B199" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="200" customHeight="1" spans="1:2">
+      <c r="A200" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="B200" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="201" customHeight="1" spans="1:2">
+      <c r="A201" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="B201" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="202" customHeight="1" spans="1:2">
+      <c r="A202" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="B202" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="203" customHeight="1" spans="1:2">
+      <c r="A203" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="B203" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="204" customHeight="1" spans="1:2">
+      <c r="A204" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="B204" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="205" customHeight="1" spans="1:2">
+      <c r="A205" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="B205" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="206" customHeight="1" spans="1:2">
+      <c r="A206" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="B206" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="207" customHeight="1" spans="1:2">
+      <c r="A207" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="B207" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="208" customHeight="1" spans="1:2">
+      <c r="A208" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B208" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="209" customHeight="1" spans="1:2">
+      <c r="A209" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="B209" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="210" customHeight="1" spans="1:2">
+      <c r="A210" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="B210" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="211" customHeight="1" spans="1:2">
+      <c r="A211" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="B211" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="212" customHeight="1" spans="1:2">
+      <c r="A212" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="B212" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="213" customHeight="1" spans="1:2">
+      <c r="A213" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="B213" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="214" customHeight="1" spans="1:2">
+      <c r="A214" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="B214" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="215" customHeight="1" spans="1:2">
+      <c r="A215" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="B215" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="216" customHeight="1" spans="1:2">
+      <c r="A216" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="B216" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="217" customHeight="1" spans="1:2">
+      <c r="A217" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="B217" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="218" customHeight="1" spans="1:2">
+      <c r="A218" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="B218" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="219" customHeight="1" spans="1:2">
+      <c r="A219" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="B219" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="220" customHeight="1" spans="1:2">
+      <c r="A220" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="B220" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="221" customHeight="1" spans="1:2">
+      <c r="A221" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="B221" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="222" customHeight="1" spans="1:2">
+      <c r="A222" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="B222" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="223" customHeight="1" spans="1:2">
+      <c r="A223" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="B223" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="224" customHeight="1" spans="1:2">
+      <c r="A224" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="B224" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="225" customHeight="1" spans="1:2">
+      <c r="A225" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="B225" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="226" customHeight="1" spans="1:2">
+      <c r="A226" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="B226" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="227" customHeight="1" spans="1:2">
+      <c r="A227" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="B227" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="228" customHeight="1" spans="1:2">
+      <c r="A228" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="B228" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="229" customHeight="1" spans="1:2">
+      <c r="A229" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="B229" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="230" customHeight="1" spans="1:2">
+      <c r="A230" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="B230" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="231" customHeight="1" spans="1:2">
+      <c r="A231" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="B231" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="232" customHeight="1" spans="1:2">
+      <c r="A232" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="B232" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="233" customHeight="1" spans="1:2">
+      <c r="A233" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="B233" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="234" customHeight="1" spans="1:2">
+      <c r="A234" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="B234" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="235" customHeight="1" spans="1:2">
+      <c r="A235" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="B235" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="236" customHeight="1" spans="1:2">
+      <c r="A236" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="B236" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="237" customHeight="1" spans="1:2">
+      <c r="A237" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="B237" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="238" customHeight="1" spans="1:2">
+      <c r="A238" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="B238" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="239" customHeight="1" spans="1:2">
+      <c r="A239" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="B239" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="240" customHeight="1" spans="1:2">
+      <c r="A240" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="B240" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="241" customHeight="1" spans="1:2">
+      <c r="A241" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="B241" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="242" customHeight="1" spans="1:2">
+      <c r="A242" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="B242" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="243" customHeight="1" spans="1:2">
+      <c r="A243" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="B243" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="244" customHeight="1" spans="1:2">
+      <c r="A244" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="B244" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="245" customHeight="1" spans="1:2">
+      <c r="A245" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="B245" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="246" customHeight="1" spans="1:2">
+      <c r="A246" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="B246" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="247" customHeight="1" spans="1:2">
+      <c r="A247" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="B247" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="248" customHeight="1" spans="1:2">
+      <c r="A248" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="B248" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="249" customHeight="1" spans="1:2">
+      <c r="A249" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="B249" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="250" customHeight="1" spans="1:2">
+      <c r="A250" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="B250" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="251" customHeight="1" spans="1:2">
+      <c r="A251" s="4" t="s">
+        <v>258</v>
+      </c>
+      <c r="B251" s="4" t="s">
+        <v>209</v>
       </c>
     </row>
   </sheetData>
@@ -3071,11 +4077,11 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:E1000"/>
-  <sheetFormatPr defaultColWidth="12.6296296296296" defaultRowHeight="15.75" customHeight="1" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="12.6285714285714" defaultRowHeight="15.75" customHeight="1" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="72.3796296296296" customWidth="1"/>
-    <col min="2" max="2" width="11.25" customWidth="1"/>
-    <col min="3" max="4" width="44.75" customWidth="1"/>
+    <col min="1" max="1" width="72.3809523809524" customWidth="1"/>
+    <col min="2" max="2" width="11.247619047619" customWidth="1"/>
+    <col min="3" max="4" width="44.752380952381" customWidth="1"/>
     <col min="5" max="5" width="31" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3084,10 +4090,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>174</v>
+        <v>259</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>175</v>
+        <v>260</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>2</v>
@@ -3104,13 +4110,13 @@
         <v>5</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>176</v>
+        <v>261</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="3" customHeight="1" spans="1:5">
+    <row r="3" customHeight="1" spans="1:4">
       <c r="A3" s="1" t="s">
         <v>108</v>
       </c>
@@ -3119,7 +4125,7 @@
       </c>
       <c r="D3" s="2"/>
     </row>
-    <row r="4" customHeight="1" spans="1:5">
+    <row r="4" customHeight="1" spans="1:4">
       <c r="A4" s="1" t="s">
         <v>109</v>
       </c>
@@ -3128,7 +4134,7 @@
       </c>
       <c r="D4" s="2"/>
     </row>
-    <row r="5" customHeight="1" spans="1:5">
+    <row r="5" customHeight="1" spans="1:4">
       <c r="A5" s="1" t="s">
         <v>110</v>
       </c>
@@ -3137,7 +4143,7 @@
       </c>
       <c r="D5" s="2"/>
     </row>
-    <row r="6" customHeight="1" spans="1:5">
+    <row r="6" customHeight="1" spans="1:4">
       <c r="A6" s="1" t="s">
         <v>111</v>
       </c>
@@ -3146,7 +4152,7 @@
       </c>
       <c r="D6" s="2"/>
     </row>
-    <row r="7" customHeight="1" spans="1:5">
+    <row r="7" customHeight="1" spans="1:4">
       <c r="A7" s="1" t="s">
         <v>112</v>
       </c>
@@ -3155,7 +4161,7 @@
       </c>
       <c r="D7" s="2"/>
     </row>
-    <row r="8" customHeight="1" spans="1:5">
+    <row r="8" customHeight="1" spans="1:4">
       <c r="A8" s="1" t="s">
         <v>113</v>
       </c>
@@ -3164,7 +4170,7 @@
       </c>
       <c r="D8" s="2"/>
     </row>
-    <row r="9" customHeight="1" spans="1:5">
+    <row r="9" customHeight="1" spans="1:4">
       <c r="A9" s="1" t="s">
         <v>114</v>
       </c>
@@ -3173,7 +4179,7 @@
       </c>
       <c r="D9" s="2"/>
     </row>
-    <row r="10" customHeight="1" spans="1:5">
+    <row r="10" customHeight="1" spans="1:4">
       <c r="A10" s="1" t="s">
         <v>115</v>
       </c>
@@ -3181,11 +4187,11 @@
         <v>3</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>177</v>
+        <v>262</v>
       </c>
       <c r="D10" s="2"/>
     </row>
-    <row r="11" customHeight="1" spans="1:5">
+    <row r="11" customHeight="1" spans="1:4">
       <c r="A11" s="1" t="s">
         <v>116</v>
       </c>
@@ -3194,7 +4200,7 @@
       </c>
       <c r="D11" s="2"/>
     </row>
-    <row r="12" customHeight="1" spans="1:5">
+    <row r="12" customHeight="1" spans="1:4">
       <c r="A12" s="1" t="s">
         <v>117</v>
       </c>
@@ -3203,7 +4209,7 @@
       </c>
       <c r="D12" s="2"/>
     </row>
-    <row r="13" customHeight="1" spans="1:5">
+    <row r="13" customHeight="1" spans="1:4">
       <c r="A13" s="1" t="s">
         <v>118</v>
       </c>
@@ -3212,7 +4218,7 @@
       </c>
       <c r="D13" s="2"/>
     </row>
-    <row r="14" customHeight="1" spans="1:5">
+    <row r="14" customHeight="1" spans="1:4">
       <c r="A14" s="1" t="s">
         <v>119</v>
       </c>
@@ -3221,7 +4227,7 @@
       </c>
       <c r="D14" s="2"/>
     </row>
-    <row r="15" customHeight="1" spans="1:5">
+    <row r="15" customHeight="1" spans="1:4">
       <c r="A15" s="1" t="s">
         <v>120</v>
       </c>
@@ -3230,7 +4236,7 @@
       </c>
       <c r="D15" s="2"/>
     </row>
-    <row r="16" customHeight="1" spans="1:5">
+    <row r="16" customHeight="1" spans="1:4">
       <c r="A16" s="1" t="s">
         <v>121</v>
       </c>
@@ -3292,7 +4298,7 @@
         <v>4</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>178</v>
+        <v>263</v>
       </c>
       <c r="D22" s="2"/>
     </row>
@@ -3304,7 +4310,7 @@
         <v>4</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>179</v>
+        <v>264</v>
       </c>
       <c r="D23" s="2"/>
     </row>
@@ -3334,7 +4340,7 @@
         <v>4</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>180</v>
+        <v>265</v>
       </c>
       <c r="D26" s="2"/>
     </row>
@@ -3346,7 +4352,7 @@
         <v>3</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>181</v>
+        <v>266</v>
       </c>
       <c r="D27" s="2"/>
     </row>
@@ -3376,7 +4382,7 @@
         <v>4</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>182</v>
+        <v>267</v>
       </c>
       <c r="D30" s="2"/>
     </row>
@@ -3397,7 +4403,7 @@
         <v>4</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>183</v>
+        <v>268</v>
       </c>
       <c r="D32" s="2"/>
     </row>
@@ -3463,7 +4469,7 @@
         <v>4</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>184</v>
+        <v>269</v>
       </c>
       <c r="D39" s="2"/>
     </row>
@@ -3484,7 +4490,7 @@
         <v>3</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>185</v>
+        <v>270</v>
       </c>
       <c r="D41" s="2"/>
     </row>
@@ -3532,7 +4538,7 @@
         <v>5</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>186</v>
+        <v>271</v>
       </c>
       <c r="D46" s="2"/>
     </row>
@@ -3571,152 +4577,152 @@
         <v>5</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>187</v>
+        <v>272</v>
       </c>
       <c r="D50" s="2"/>
     </row>
     <row r="51" customHeight="1" spans="1:4">
       <c r="A51" s="1" t="s">
-        <v>156</v>
+        <v>273</v>
       </c>
       <c r="D51" s="2"/>
     </row>
     <row r="52" customHeight="1" spans="1:4">
       <c r="A52" s="1" t="s">
-        <v>157</v>
+        <v>274</v>
       </c>
       <c r="D52" s="2"/>
     </row>
     <row r="53" customHeight="1" spans="1:4">
       <c r="A53" s="1" t="s">
-        <v>158</v>
+        <v>275</v>
       </c>
       <c r="D53" s="2"/>
     </row>
     <row r="54" customHeight="1" spans="1:4">
       <c r="A54" s="1" t="s">
-        <v>159</v>
+        <v>276</v>
       </c>
       <c r="D54" s="2"/>
     </row>
     <row r="55" customHeight="1" spans="1:4">
       <c r="A55" s="1" t="s">
-        <v>160</v>
+        <v>277</v>
       </c>
       <c r="D55" s="2"/>
     </row>
     <row r="56" customHeight="1" spans="1:4">
       <c r="A56" s="1" t="s">
-        <v>161</v>
+        <v>278</v>
       </c>
       <c r="D56" s="2"/>
     </row>
     <row r="57" customHeight="1" spans="1:4">
       <c r="A57" s="1" t="s">
-        <v>162</v>
+        <v>279</v>
       </c>
       <c r="D57" s="2"/>
     </row>
     <row r="58" customHeight="1" spans="1:4">
       <c r="A58" s="1" t="s">
-        <v>163</v>
+        <v>280</v>
       </c>
       <c r="D58" s="2"/>
     </row>
     <row r="59" customHeight="1" spans="1:4">
       <c r="A59" s="1" t="s">
-        <v>164</v>
+        <v>281</v>
       </c>
       <c r="D59" s="2"/>
     </row>
     <row r="60" customHeight="1" spans="1:4">
       <c r="A60" s="1" t="s">
-        <v>165</v>
+        <v>282</v>
       </c>
       <c r="D60" s="2"/>
     </row>
     <row r="61" customHeight="1" spans="1:4">
       <c r="A61" s="1" t="s">
-        <v>166</v>
+        <v>283</v>
       </c>
       <c r="D61" s="2"/>
     </row>
     <row r="62" customHeight="1" spans="1:4">
       <c r="A62" s="1" t="s">
-        <v>167</v>
+        <v>284</v>
       </c>
       <c r="D62" s="2"/>
     </row>
     <row r="63" customHeight="1" spans="1:4">
       <c r="A63" s="1" t="s">
-        <v>168</v>
+        <v>285</v>
       </c>
       <c r="D63" s="2"/>
     </row>
     <row r="64" customHeight="1" spans="1:4">
       <c r="A64" s="1" t="s">
-        <v>169</v>
+        <v>286</v>
       </c>
       <c r="D64" s="2"/>
     </row>
     <row r="65" customHeight="1" spans="1:4">
       <c r="A65" s="1" t="s">
-        <v>170</v>
+        <v>287</v>
       </c>
       <c r="D65" s="2"/>
     </row>
     <row r="66" customHeight="1" spans="1:4">
       <c r="A66" s="1" t="s">
-        <v>171</v>
+        <v>288</v>
       </c>
       <c r="D66" s="2"/>
     </row>
     <row r="67" customHeight="1" spans="1:4">
       <c r="A67" s="1" t="s">
-        <v>172</v>
+        <v>289</v>
       </c>
       <c r="D67" s="2"/>
     </row>
     <row r="68" customHeight="1" spans="1:4">
       <c r="A68" s="1" t="s">
-        <v>173</v>
+        <v>156</v>
       </c>
       <c r="D68" s="2"/>
     </row>
-    <row r="69" customHeight="1" spans="1:4">
+    <row r="69" customHeight="1" spans="4:4">
       <c r="D69" s="2"/>
     </row>
-    <row r="70" customHeight="1" spans="1:4">
+    <row r="70" customHeight="1" spans="4:4">
       <c r="D70" s="2"/>
     </row>
-    <row r="71" customHeight="1" spans="1:4">
+    <row r="71" customHeight="1" spans="4:4">
       <c r="D71" s="2"/>
     </row>
-    <row r="72" customHeight="1" spans="1:4">
+    <row r="72" customHeight="1" spans="4:4">
       <c r="D72" s="2"/>
     </row>
-    <row r="73" customHeight="1" spans="1:4">
+    <row r="73" customHeight="1" spans="4:4">
       <c r="D73" s="2"/>
     </row>
-    <row r="74" customHeight="1" spans="1:4">
+    <row r="74" customHeight="1" spans="4:4">
       <c r="D74" s="2"/>
     </row>
-    <row r="75" customHeight="1" spans="1:4">
+    <row r="75" customHeight="1" spans="4:4">
       <c r="D75" s="2"/>
     </row>
-    <row r="76" customHeight="1" spans="1:4">
+    <row r="76" customHeight="1" spans="4:4">
       <c r="D76" s="2"/>
     </row>
-    <row r="77" customHeight="1" spans="1:4">
+    <row r="77" customHeight="1" spans="4:4">
       <c r="D77" s="2"/>
     </row>
-    <row r="78" customHeight="1" spans="1:4">
+    <row r="78" customHeight="1" spans="4:4">
       <c r="D78" s="2"/>
     </row>
-    <row r="79" customHeight="1" spans="1:4">
+    <row r="79" customHeight="1" spans="4:4">
       <c r="D79" s="2"/>
     </row>
-    <row r="80" customHeight="1" spans="1:4">
+    <row r="80" customHeight="1" spans="4:4">
       <c r="D80" s="2"/>
     </row>
     <row r="81" customHeight="1" spans="4:4">

</xml_diff>